<commit_message>
Modified docs/Sales_Data_Dictionary.xlsx and added docs/ETL_Process.xlsx with new ETL steps
</commit_message>
<xml_diff>
--- a/docs/Sales_Data_Dictionary.xlsx
+++ b/docs/Sales_Data_Dictionary.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Samira\Data\Projects\Syntecxhub Internship\1. Week\Sales_Performance_Dashboard\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D31417A-2A20-425C-8439-AAF4B09C4646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54DC45C3-AB0E-44F9-A70C-08D235907519}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{85312015-592B-44E7-A4EB-E2F6F45D90B6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="3" xr2:uid="{85312015-592B-44E7-A4EB-E2F6F45D90B6}"/>
   </bookViews>
   <sheets>
     <sheet name="Schema" sheetId="1" r:id="rId1"/>
     <sheet name="Explanation" sheetId="2" r:id="rId2"/>
     <sheet name="Measurments" sheetId="3" r:id="rId3"/>
+    <sheet name="Reference Tables" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="260">
   <si>
     <t>Column Name</t>
   </si>
@@ -1245,6 +1246,54 @@
       </rPr>
       <t xml:space="preserve"> grouped by Ship Mode</t>
     </r>
+  </si>
+  <si>
+    <t>Reference Table</t>
+  </si>
+  <si>
+    <t>Source Column</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>DimDate</t>
+  </si>
+  <si>
+    <t>Time Intelligence</t>
+  </si>
+  <si>
+    <t>DimCustomer</t>
+  </si>
+  <si>
+    <t>Customer Analysis</t>
+  </si>
+  <si>
+    <t>DimProduct</t>
+  </si>
+  <si>
+    <t>DimCategory</t>
+  </si>
+  <si>
+    <t>Category, Sub-Category</t>
+  </si>
+  <si>
+    <t>DimGeography</t>
+  </si>
+  <si>
+    <t>Country, State, City, Region</t>
+  </si>
+  <si>
+    <t>DimShipMode</t>
+  </si>
+  <si>
+    <t>Shipment Analysis</t>
+  </si>
+  <si>
+    <t>DimPaymentMode</t>
+  </si>
+  <si>
+    <t>Payment Analysis</t>
   </si>
 </sst>
 </file>
@@ -1318,7 +1367,38 @@
   <cellStyles count="1">
     <cellStyle name="عادي" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="22">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="left" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1431,15 +1511,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A18F2AFC-10A3-4738-B279-9AC757BAD61F}" name="الجدول1" displayName="الجدول1" ref="A1:F30" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A18F2AFC-10A3-4738-B279-9AC757BAD61F}" name="الجدول1" displayName="الجدول1" ref="A1:F30" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
   <autoFilter ref="A1:F30" xr:uid="{A18F2AFC-10A3-4738-B279-9AC757BAD61F}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{46AC1AEF-9A80-43FA-8BE0-F10CAE79E2DB}" name="Column Name" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{399EF6DA-4484-4039-8F4D-4E62C7BDA8F0}" name="Description" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{535B9255-1105-4D10-B51E-C6C786243CC3}" name="Data Type" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{660B9155-8D46-4F98-A2D6-434C852CE424}" name="Category" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{459799EB-09EA-4A07-84EF-EC18B7BA44BE}" name="Source" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{8B1B420D-F3B2-476C-A21D-484DDC01E455}" name="Example" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{46AC1AEF-9A80-43FA-8BE0-F10CAE79E2DB}" name="Column Name" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{399EF6DA-4484-4039-8F4D-4E62C7BDA8F0}" name="Description" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{535B9255-1105-4D10-B51E-C6C786243CC3}" name="Data Type" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{660B9155-8D46-4F98-A2D6-434C852CE424}" name="Category" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{459799EB-09EA-4A07-84EF-EC18B7BA44BE}" name="Source" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{8B1B420D-F3B2-476C-A21D-484DDC01E455}" name="Example" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1449,7 +1529,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6FAC286D-A874-4ED0-B2AF-F03932A04B79}" name="الجدول2" displayName="الجدول2" ref="A1:B4" totalsRowShown="0">
   <autoFilter ref="A1:B4" xr:uid="{6FAC286D-A874-4ED0-B2AF-F03932A04B79}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{F25EBA2B-0E30-4288-B5DB-99589D3D13F2}" name="Category" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{F25EBA2B-0E30-4288-B5DB-99589D3D13F2}" name="Category" dataDxfId="13"/>
     <tableColumn id="2" xr3:uid="{173FCAF8-E2F6-4419-BBDC-4C0678F58625}" name="Explanation"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1457,15 +1537,27 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F8B86951-948D-4708-90A4-CEB49F0431D2}" name="الجدول3" displayName="الجدول3" ref="A1:F46" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F8B86951-948D-4708-90A4-CEB49F0431D2}" name="الجدول3" displayName="الجدول3" ref="A1:F46" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
   <autoFilter ref="A1:F46" xr:uid="{F8B86951-948D-4708-90A4-CEB49F0431D2}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{93B471AF-061A-49AC-9CFB-65A81042FB10}" name="Measure / KPI" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{3AD3B45A-EB6C-4162-8BB0-06DC52222794}" name="Business Purpose" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{10E9063B-32F1-4E90-AF89-B409D19D6AA0}" name="Formula / Logic" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{C682141D-D63B-4A21-B8A3-DCD77098432C}" name="KPI Category" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{492AE4AF-C28A-4630-BC75-9ED55EF73DB5}" name="Format" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{70F76F97-0D47-4F8F-845D-8411DD205FA6}" name="Implementation Method" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{93B471AF-061A-49AC-9CFB-65A81042FB10}" name="Measure / KPI" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{3AD3B45A-EB6C-4162-8BB0-06DC52222794}" name="Business Purpose" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{10E9063B-32F1-4E90-AF89-B409D19D6AA0}" name="Formula / Logic" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{C682141D-D63B-4A21-B8A3-DCD77098432C}" name="KPI Category" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{492AE4AF-C28A-4630-BC75-9ED55EF73DB5}" name="Format" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{70F76F97-0D47-4F8F-845D-8411DD205FA6}" name="Implementation Method" dataDxfId="5"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{5E8F4507-31C3-4F3D-9503-568D32610F06}" name="الجدول4" displayName="الجدول4" ref="A1:C8" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <autoFilter ref="A1:C8" xr:uid="{5E8F4507-31C3-4F3D-9503-568D32610F06}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{D21DE232-CBB4-4537-AC43-63EE14DF2D32}" name="Reference Table" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{3D2EE634-8B76-4752-B902-87690304721E}" name="Source Column" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{2E02C6D4-489C-4286-B611-B914CD3CAEC0}" name="Purpose" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3372,4 +3464,111 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB85D823-EAC3-48CE-A103-DF088C2939C7}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>259</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Completed Phase 5 DAX development and updated ETL process tracker
</commit_message>
<xml_diff>
--- a/docs/Sales_Data_Dictionary.xlsx
+++ b/docs/Sales_Data_Dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Samira\Data\Projects\Syntecxhub Internship\1. Week\Sales_Performance_Dashboard\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54DC45C3-AB0E-44F9-A70C-08D235907519}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82A7FA8B-8E5C-4AB5-BF8F-C2850F39AC92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="3" xr2:uid="{85312015-592B-44E7-A4EB-E2F6F45D90B6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" activeTab="2" xr2:uid="{85312015-592B-44E7-A4EB-E2F6F45D90B6}"/>
   </bookViews>
   <sheets>
     <sheet name="Schema" sheetId="1" r:id="rId1"/>
@@ -1322,12 +1322,18 @@
       <name val="Arial Unicode MS"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -1342,7 +1348,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1363,11 +1369,26 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="عادي" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="22">
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -1386,18 +1407,6 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="left" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1539,6 +1548,9 @@
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F8B86951-948D-4708-90A4-CEB49F0431D2}" name="الجدول3" displayName="الجدول3" ref="A1:F46" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
   <autoFilter ref="A1:F46" xr:uid="{F8B86951-948D-4708-90A4-CEB49F0431D2}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F17">
+    <sortCondition ref="E1:E46"/>
+  </sortState>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{93B471AF-061A-49AC-9CFB-65A81042FB10}" name="Measure / KPI" dataDxfId="10"/>
     <tableColumn id="2" xr3:uid="{3AD3B45A-EB6C-4162-8BB0-06DC52222794}" name="Business Purpose" dataDxfId="9"/>
@@ -1552,12 +1564,12 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{5E8F4507-31C3-4F3D-9503-568D32610F06}" name="الجدول4" displayName="الجدول4" ref="A1:C8" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{5E8F4507-31C3-4F3D-9503-568D32610F06}" name="الجدول4" displayName="الجدول4" ref="A1:C8" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
   <autoFilter ref="A1:C8" xr:uid="{5E8F4507-31C3-4F3D-9503-568D32610F06}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{D21DE232-CBB4-4537-AC43-63EE14DF2D32}" name="Reference Table" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{3D2EE634-8B76-4752-B902-87690304721E}" name="Source Column" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{2E02C6D4-489C-4286-B611-B914CD3CAEC0}" name="Purpose" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{D21DE232-CBB4-4537-AC43-63EE14DF2D32}" name="Reference Table" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{3D2EE634-8B76-4752-B902-87690304721E}" name="Source Column" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{2E02C6D4-489C-4286-B611-B914CD3CAEC0}" name="Purpose" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1861,14 +1873,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E773590-3DD3-4687-9120-A619F464FC79}">
   <dimension ref="A1:F30"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="45.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1891,7 +1903,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="28.8">
+    <row r="2" spans="1:6" ht="30">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1911,7 +1923,7 @@
         <v>4407</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="28.8">
+    <row r="3" spans="1:6" ht="30">
       <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
@@ -1951,7 +1963,7 @@
         <v>43789</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" ht="30">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
@@ -1971,7 +1983,7 @@
         <v>43794</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" ht="30">
       <c r="A6" s="2" t="s">
         <v>21</v>
       </c>
@@ -2011,7 +2023,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" ht="30">
       <c r="A8" s="2" t="s">
         <v>27</v>
       </c>
@@ -2051,7 +2063,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" ht="30">
       <c r="A10" s="2" t="s">
         <v>33</v>
       </c>
@@ -2131,7 +2143,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="28.8">
+    <row r="14" spans="1:6" ht="30">
       <c r="A14" s="2" t="s">
         <v>45</v>
       </c>
@@ -2151,7 +2163,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="28.8">
+    <row r="15" spans="1:6" ht="30">
       <c r="A15" s="2" t="s">
         <v>3</v>
       </c>
@@ -2211,7 +2223,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" ht="30">
       <c r="A18" s="2" t="s">
         <v>56</v>
       </c>
@@ -2251,7 +2263,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" ht="30">
       <c r="A20" s="2" t="s">
         <v>62</v>
       </c>
@@ -2271,7 +2283,7 @@
         <v>150.98400000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="28.8">
+    <row r="21" spans="1:6" ht="30">
       <c r="A21" s="2" t="s">
         <v>64</v>
       </c>
@@ -2311,7 +2323,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" ht="30">
       <c r="A23" s="2" t="s">
         <v>69</v>
       </c>
@@ -2331,7 +2343,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" ht="30">
       <c r="A24" s="2" t="s">
         <v>72</v>
       </c>
@@ -2351,7 +2363,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="28.8">
+    <row r="25" spans="1:6" ht="30">
       <c r="A25" s="2" t="s">
         <v>75</v>
       </c>
@@ -2371,7 +2383,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" ht="30">
       <c r="A26" s="2" t="s">
         <v>77</v>
       </c>
@@ -2391,7 +2403,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" ht="30">
       <c r="A27" s="2" t="s">
         <v>80</v>
       </c>
@@ -2411,7 +2423,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" ht="30">
       <c r="A28" s="2" t="s">
         <v>82</v>
       </c>
@@ -2431,7 +2443,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" ht="30">
       <c r="A29" s="2" t="s">
         <v>85</v>
       </c>
@@ -2451,7 +2463,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="28.8">
+    <row r="30" spans="1:6" ht="30">
       <c r="A30" s="2" t="s">
         <v>87</v>
       </c>
@@ -2482,7 +2494,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6DEB35F-CE02-426F-A567-FCF45D1310E9}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
@@ -2527,13 +2539,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4F48300-13CA-466B-B82B-283F76F5825A}">
   <dimension ref="A1:F46"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="51.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="51.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2558,7 +2570,7 @@
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="8" t="s">
         <v>98</v>
       </c>
       <c r="B2" s="6" t="s">
@@ -2578,7 +2590,7 @@
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="8" t="s">
         <v>103</v>
       </c>
       <c r="B3" s="6" t="s">
@@ -2597,98 +2609,98 @@
         <v>154</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="28.8">
-      <c r="A4" s="6" t="s">
-        <v>106</v>
+    <row r="4" spans="1:6" ht="30">
+      <c r="A4" s="8" t="s">
+        <v>120</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>107</v>
+        <v>155</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>108</v>
+        <v>156</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>101</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>8</v>
+        <v>102</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="28.8">
-      <c r="A5" s="6" t="s">
-        <v>109</v>
+    <row r="5" spans="1:6" ht="30">
+      <c r="A5" s="8" t="s">
+        <v>121</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>110</v>
+        <v>157</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>111</v>
+        <v>158</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>8</v>
+        <v>102</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="28.8">
-      <c r="A6" s="6" t="s">
-        <v>113</v>
+    <row r="6" spans="1:6" ht="30">
+      <c r="A6" s="8" t="s">
+        <v>122</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>114</v>
+        <v>159</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>115</v>
+        <v>160</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>8</v>
+        <v>102</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="28.8">
-      <c r="A7" s="6" t="s">
-        <v>117</v>
+    <row r="7" spans="1:6" ht="30">
+      <c r="A7" s="8" t="s">
+        <v>123</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>118</v>
+        <v>161</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>119</v>
+        <v>162</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>8</v>
+        <v>102</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="28.8">
-      <c r="A8" s="6" t="s">
-        <v>120</v>
+    <row r="8" spans="1:6" ht="25.5">
+      <c r="A8" s="8" t="s">
+        <v>131</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>155</v>
+        <v>170</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>156</v>
+        <v>171</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>101</v>
+        <v>128</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>102</v>
@@ -2697,118 +2709,118 @@
         <v>154</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
-      <c r="A9" s="6" t="s">
-        <v>121</v>
+    <row r="9" spans="1:6" ht="30">
+      <c r="A9" s="8" t="s">
+        <v>124</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>102</v>
+        <v>58</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="28.8">
-      <c r="A10" s="6" t="s">
-        <v>122</v>
+    <row r="10" spans="1:6" ht="30">
+      <c r="A10" s="8" t="s">
+        <v>165</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>159</v>
+        <v>125</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>102</v>
+        <v>126</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="28.8">
-      <c r="A11" s="6" t="s">
-        <v>123</v>
+    <row r="11" spans="1:6" ht="30">
+      <c r="A11" s="8" t="s">
+        <v>168</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>161</v>
+        <v>127</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>102</v>
+        <v>126</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="28.8">
-      <c r="A12" s="6" t="s">
-        <v>124</v>
+    <row r="12" spans="1:6" ht="30">
+      <c r="A12" s="8" t="s">
+        <v>172</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>163</v>
+        <v>132</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>58</v>
+        <v>126</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="28.8">
-      <c r="A13" s="6" t="s">
-        <v>165</v>
+    <row r="13" spans="1:6" ht="30">
+      <c r="A13" s="8" t="s">
+        <v>106</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>166</v>
+        <v>108</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>101</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>126</v>
+        <v>8</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="28.8">
-      <c r="A14" s="6" t="s">
-        <v>129</v>
+    <row r="14" spans="1:6" ht="30">
+      <c r="A14" s="8" t="s">
+        <v>109</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>167</v>
+        <v>111</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>128</v>
+        <v>112</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>8</v>
@@ -2817,61 +2829,61 @@
         <v>154</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="28.8">
-      <c r="A15" s="6" t="s">
-        <v>168</v>
+    <row r="15" spans="1:6" ht="30">
+      <c r="A15" s="8" t="s">
+        <v>113</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>169</v>
+        <v>115</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>126</v>
+        <v>8</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="26.4">
-      <c r="A16" s="6" t="s">
-        <v>131</v>
+    <row r="16" spans="1:6" ht="30">
+      <c r="A16" s="8" t="s">
+        <v>117</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>170</v>
+        <v>118</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>171</v>
+        <v>119</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>102</v>
+        <v>8</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="28.8">
-      <c r="A17" s="6" t="s">
-        <v>172</v>
+    <row r="17" spans="1:6" ht="30">
+      <c r="A17" s="8" t="s">
+        <v>129</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>128</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>126</v>
+        <v>8</v>
       </c>
       <c r="F17" s="6" t="s">
         <v>154</v>
@@ -3057,7 +3069,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" ht="30">
       <c r="A27" s="6" t="s">
         <v>141</v>
       </c>
@@ -3077,7 +3089,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" ht="30">
       <c r="A28" s="6" t="s">
         <v>142</v>
       </c>
@@ -3097,7 +3109,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="28.8">
+    <row r="29" spans="1:6" ht="30">
       <c r="A29" s="6" t="s">
         <v>147</v>
       </c>
@@ -3117,7 +3129,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="28.8">
+    <row r="30" spans="1:6" ht="30">
       <c r="A30" s="6" t="s">
         <v>200</v>
       </c>
@@ -3137,7 +3149,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="28.8">
+    <row r="31" spans="1:6" ht="30">
       <c r="A31" s="6" t="s">
         <v>133</v>
       </c>
@@ -3157,7 +3169,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="28.8">
+    <row r="32" spans="1:6" ht="30">
       <c r="A32" s="6" t="s">
         <v>134</v>
       </c>
@@ -3177,7 +3189,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="28.8">
+    <row r="33" spans="1:6" ht="30">
       <c r="A33" s="6" t="s">
         <v>139</v>
       </c>
@@ -3197,7 +3209,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="28.8">
+    <row r="34" spans="1:6" ht="30">
       <c r="A34" s="6" t="s">
         <v>210</v>
       </c>
@@ -3237,7 +3249,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" ht="30">
       <c r="A36" s="6" t="s">
         <v>216</v>
       </c>
@@ -3257,7 +3269,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="28.8">
+    <row r="37" spans="1:6" ht="30">
       <c r="A37" s="6" t="s">
         <v>219</v>
       </c>
@@ -3277,7 +3289,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="28.8">
+    <row r="38" spans="1:6" ht="30">
       <c r="A38" s="6" t="s">
         <v>222</v>
       </c>
@@ -3297,7 +3309,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="28.8">
+    <row r="39" spans="1:6" ht="30">
       <c r="A39" s="6" t="s">
         <v>225</v>
       </c>
@@ -3317,7 +3329,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" spans="1:6" ht="30">
       <c r="A40" s="6" t="s">
         <v>228</v>
       </c>
@@ -3337,7 +3349,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="28.8">
+    <row r="41" spans="1:6" ht="30">
       <c r="A41" s="6" t="s">
         <v>230</v>
       </c>
@@ -3357,7 +3369,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="28.8">
+    <row r="42" spans="1:6" ht="30">
       <c r="A42" s="6" t="s">
         <v>143</v>
       </c>
@@ -3377,7 +3389,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="28.8">
+    <row r="43" spans="1:6" ht="30">
       <c r="A43" s="6" t="s">
         <v>144</v>
       </c>
@@ -3397,7 +3409,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="28.8">
+    <row r="44" spans="1:6" ht="30">
       <c r="A44" s="6" t="s">
         <v>237</v>
       </c>
@@ -3417,7 +3429,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="45" spans="1:6">
+    <row r="45" spans="1:6" ht="30">
       <c r="A45" s="6" t="s">
         <v>146</v>
       </c>
@@ -3437,7 +3449,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="46" spans="1:6">
+    <row r="46" spans="1:6" ht="30">
       <c r="A46" s="6" t="s">
         <v>145</v>
       </c>
@@ -3469,12 +3481,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB85D823-EAC3-48CE-A103-DF088C2939C7}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.6640625" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3488,7 +3500,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" ht="30">
       <c r="A2" s="6" t="s">
         <v>247</v>
       </c>
@@ -3499,7 +3511,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" ht="30">
       <c r="A3" s="6" t="s">
         <v>249</v>
       </c>
@@ -3521,7 +3533,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" ht="30">
       <c r="A5" s="6" t="s">
         <v>252</v>
       </c>
@@ -3532,7 +3544,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" ht="30">
       <c r="A6" s="6" t="s">
         <v>254</v>
       </c>
@@ -3543,7 +3555,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" ht="30">
       <c r="A7" s="6" t="s">
         <v>256</v>
       </c>
@@ -3554,7 +3566,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" ht="30">
       <c r="A8" s="6" t="s">
         <v>258</v>
       </c>

</xml_diff>